<commit_message>
correct employee payload to include usergroup
</commit_message>
<xml_diff>
--- a/Mapping.xlsx
+++ b/Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nanfung-my.sharepoint.com/personal/rayland_cheng_nanfung_com/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{31AA260D-4F95-4752-A820-07BFBF0D81CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DF600C53-2015-4D01-9E24-636BD37A67B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Department" sheetId="2" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="212">
   <si>
     <t>處編號</t>
   </si>
@@ -725,18 +725,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -757,7 +751,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -765,7 +759,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1104,7 +1097,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G65"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.6"/>
   <cols>
     <col min="1" max="1" width="15.28515625" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.85546875" style="1" customWidth="1"/>
@@ -1113,7 +1106,8 @@
     <col min="5" max="5" width="9.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="10" style="1" customWidth="1"/>
     <col min="7" max="7" width="55.42578125" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="8" max="8" width="17.85546875" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -1136,7 +1130,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" ht="12.95">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1178,7 +1172,7 @@
       <c r="F3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="1" t="s">
@@ -1220,7 +1214,9 @@
       <c r="F5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="4"/>
+      <c r="G5" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="1" t="s">
@@ -1241,7 +1237,9 @@
       <c r="F6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="4"/>
+      <c r="G6" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="1" t="s">
@@ -1421,7 +1419,9 @@
       <c r="F14" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="4"/>
+      <c r="G14" s="1" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="1" t="s">
@@ -1442,7 +1442,7 @@
       <c r="F15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G15" s="5"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="1" t="s">
@@ -1642,6 +1642,7 @@
       <c r="F24" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="1" t="s">
@@ -1685,7 +1686,7 @@
       <c r="F26" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G26" s="5"/>
+      <c r="G26" s="4"/>
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="1" t="s">
@@ -1726,6 +1727,7 @@
       <c r="F28" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G28" s="4"/>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="1" t="s">
@@ -1766,6 +1768,7 @@
       <c r="F30" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G30" s="4"/>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="1" t="s">
@@ -1786,6 +1789,7 @@
       <c r="F31" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G31" s="4"/>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="1" t="s">
@@ -1806,7 +1810,7 @@
       <c r="F32" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G32" s="5"/>
+      <c r="G32" s="4"/>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="1" t="s">
@@ -1824,6 +1828,7 @@
       <c r="F33" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="1" t="s">
@@ -1867,7 +1872,7 @@
       <c r="F35" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G35" s="5"/>
+      <c r="G35" s="4"/>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="1" t="s">
@@ -1911,7 +1916,7 @@
       <c r="F37" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G37" s="5"/>
+      <c r="G37" s="4"/>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="1" t="s">
@@ -1932,6 +1937,7 @@
       <c r="F38" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G38" s="4"/>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="1" t="s">
@@ -1952,6 +1958,7 @@
       <c r="F39" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G39" s="4"/>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="1" t="s">
@@ -2130,6 +2137,7 @@
       <c r="F47" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G47" s="4"/>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="1" t="s">
@@ -2150,7 +2158,7 @@
       <c r="F48" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G48" s="5"/>
+      <c r="G48" s="4"/>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" s="1" t="s">
@@ -2194,6 +2202,7 @@
       <c r="F50" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G50" s="4"/>
     </row>
     <row r="51" spans="1:7">
       <c r="A51" s="1" t="s">
@@ -2329,7 +2338,7 @@
       <c r="F56" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G56" s="5"/>
+      <c r="G56" s="4"/>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" s="1" t="s">
@@ -2350,7 +2359,7 @@
       <c r="F57" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G57" s="5"/>
+      <c r="G57" s="4"/>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" s="1" t="s">
@@ -2371,7 +2380,9 @@
       <c r="F58" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G58" s="4"/>
+      <c r="G58" s="1" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" s="1" t="s">
@@ -2392,6 +2403,7 @@
       <c r="F59" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G59" s="4"/>
     </row>
     <row r="60" spans="1:7">
       <c r="A60" s="1" t="s">
@@ -2412,6 +2424,7 @@
       <c r="F60" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G60" s="4"/>
     </row>
     <row r="61" spans="1:7">
       <c r="A61" s="1" t="s">
@@ -2432,6 +2445,7 @@
       <c r="F61" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="G61" s="4"/>
     </row>
     <row r="62" spans="1:7">
       <c r="A62" s="1" t="s">
@@ -2493,7 +2507,7 @@
       <c r="F64" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G64" s="5"/>
+      <c r="G64" s="4"/>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" s="1" t="s">
@@ -2514,7 +2528,7 @@
       <c r="F65" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G65" s="5"/>
+      <c r="G65" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -2539,7 +2553,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320B2BF0-60F1-46AF-B517-AF44FC17F4E6}">
   <dimension ref="A1:B61"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="59.85546875" customWidth="1"/>
     <col min="2" max="2" width="59.5703125" customWidth="1"/>
@@ -2719,9 +2733,9 @@
       <c r="A20" t="s">
         <v>20</v>
       </c>
-      <c r="B20" t="e" cm="1">
+      <c r="B20" t="str" cm="1">
         <f t="array" ref="B20">INDEX(Table1[Department Name (Eng)],MATCH(Sheet1!A20,Table1[MDM Department],0),FALSE)</f>
-        <v>#N/A</v>
+        <v>AI and Data Intelligence - Properties</v>
       </c>
     </row>
     <row r="21" spans="1:2">
@@ -2737,18 +2751,18 @@
       <c r="A22" t="s">
         <v>170</v>
       </c>
-      <c r="B22" t="e" cm="1">
+      <c r="B22" t="str" cm="1">
         <f t="array" ref="B22">INDEX(Table1[Department Name (Eng)],MATCH(Sheet1!A22,Table1[MDM Department],0),FALSE)</f>
-        <v>#N/A</v>
+        <v>CHAT</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23" t="s">
         <v>47</v>
       </c>
-      <c r="B23" t="e" cm="1">
+      <c r="B23" t="str" cm="1">
         <f t="array" ref="B23">INDEX(Table1[Department Name (Eng)],MATCH(Sheet1!A23,Table1[MDM Department],0),FALSE)</f>
-        <v>#N/A</v>
+        <v>China Property</v>
       </c>
     </row>
     <row r="24" spans="1:2">
@@ -2908,9 +2922,9 @@
       <c r="A41" t="s">
         <v>25</v>
       </c>
-      <c r="B41" t="e" cm="1">
+      <c r="B41" t="str" cm="1">
         <f t="array" ref="B41">INDEX(Table1[Department Name (Eng)],MATCH(Sheet1!A41,Table1[MDM Department],0),FALSE)</f>
-        <v>#N/A</v>
+        <v>International Property</v>
       </c>
     </row>
     <row r="42" spans="1:2">

</xml_diff>